<commit_message>
Done the code for the update template
</commit_message>
<xml_diff>
--- a/src/test/resources/Templates/templateData.xlsx
+++ b/src/test/resources/Templates/templateData.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Eclipse\ICEDQ\TestGenerator\src\test\resources\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39E67149-EBBB-4F1C-9562-C6ED3D61A354}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E515B0D-542F-46CC-8C44-9F25F17AF384}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Create template" sheetId="1" r:id="rId1"/>
     <sheet name="Update template" sheetId="2" r:id="rId2"/>
+    <sheet name="Delete template" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="41">
   <si>
     <t>ruleType</t>
   </si>
@@ -118,28 +119,37 @@
     <t>updatedTemplateName</t>
   </si>
   <si>
-    <t>Compare Record Counts - Dynamic SQL_Updated</t>
-  </si>
-  <si>
-    <t>Specify Column for Diff - Full Data Compare Dynamic SQL_Updated</t>
-  </si>
-  <si>
-    <t>Data Validation - Dynamic SQL_Updated</t>
-  </si>
-  <si>
-    <t>Data Pushdown Validation - Dynamic SQL_Updated</t>
-  </si>
-  <si>
-    <t>Compare Record Counts - Import SQL_Updated</t>
-  </si>
-  <si>
-    <t>Diff and Expression based on Column Position - Import SQL_Updated</t>
-  </si>
-  <si>
-    <t>Data Validation - Import SQL_Updated</t>
-  </si>
-  <si>
-    <t>Data Pushdown Validation - Import SQL_Updated</t>
+    <t>updatedTemplateDescription</t>
+  </si>
+  <si>
+    <t>My dynamic template_Updated</t>
+  </si>
+  <si>
+    <t>My import template_Updated</t>
+  </si>
+  <si>
+    <t>My Checksum template - using dynamic template_Updated</t>
+  </si>
+  <si>
+    <t>My Recon template - using dynamic template_Updated</t>
+  </si>
+  <si>
+    <t>My Validation template - using dynamic template_Updated</t>
+  </si>
+  <si>
+    <t>My Pushdown template - using dynamic template_Updated</t>
+  </si>
+  <si>
+    <t>My Checksum template - using import template_Updated</t>
+  </si>
+  <si>
+    <t>My Recon template - using import template_Updated</t>
+  </si>
+  <si>
+    <t>My Validation template - using import template_Updated</t>
+  </si>
+  <si>
+    <t>My Pushdown template - using import template_Updated</t>
   </si>
 </sst>
 </file>
@@ -643,16 +653,17 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F7CB2AA-5EA2-492F-9BA5-269328456F4E}">
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="48.42578125" customWidth="1"/>
+    <col min="3" max="3" width="64.140625" customWidth="1"/>
     <col min="4" max="4" width="64" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="42.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>16</v>
       </c>
@@ -665,117 +676,258 @@
       <c r="D1" s="3" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>17</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="C2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>17</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D3" s="2" t="s">
+      <c r="C3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E3" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>17</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" t="s">
+        <v>35</v>
+      </c>
+      <c r="E4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>17</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>24</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" t="s">
+        <v>37</v>
+      </c>
+      <c r="E6" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>24</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C7" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" t="s">
+        <v>38</v>
+      </c>
+      <c r="E7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>24</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C8" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8" t="s">
+        <v>39</v>
+      </c>
+      <c r="E8" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>24</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D9" s="2" t="s">
+      <c r="C9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93F33FC7-11FF-4B9B-AB3B-6DD0B3697E0D}">
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16.5703125" customWidth="1"/>
+    <col min="2" max="2" width="19.7109375" customWidth="1"/>
+    <col min="3" max="3" width="59.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" t="s">
         <v>37</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>24</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" t="s">
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added a code for deletion at listing as well as details page
</commit_message>
<xml_diff>
--- a/src/test/resources/Templates/templateData.xlsx
+++ b/src/test/resources/Templates/templateData.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Eclipse\ICEDQ\TestGenerator\src\test\resources\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E515B0D-542F-46CC-8C44-9F25F17AF384}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{697D96F7-2170-4145-A950-F7BE7BD0F7CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Create template" sheetId="1" r:id="rId1"/>
     <sheet name="Update template" sheetId="2" r:id="rId2"/>
-    <sheet name="Delete template" sheetId="3" r:id="rId3"/>
+    <sheet name="Delete template - List" sheetId="3" r:id="rId3"/>
+    <sheet name="Delete template - Details" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="48">
   <si>
     <t>ruleType</t>
   </si>
@@ -150,6 +151,27 @@
   </si>
   <si>
     <t>My Pushdown template - using import template_Updated</t>
+  </si>
+  <si>
+    <t>My Checksum template - using dynamic template To delete</t>
+  </si>
+  <si>
+    <t>My Recon template - using dynamic template  To delete</t>
+  </si>
+  <si>
+    <t>My Validation template - using dynamic template  To delete</t>
+  </si>
+  <si>
+    <t>My Validation template - using import template  To delete</t>
+  </si>
+  <si>
+    <t>My Pushdown template - using import template  To delete</t>
+  </si>
+  <si>
+    <t>My dynamic template  To delete</t>
+  </si>
+  <si>
+    <t>My import template  To delete</t>
   </si>
 </sst>
 </file>
@@ -482,7 +504,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.28515625" customWidth="1"/>
@@ -643,6 +665,91 @@
       </c>
       <c r="E9" t="s">
         <v>23</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D10" t="s">
+        <v>41</v>
+      </c>
+      <c r="E10" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D11" t="s">
+        <v>42</v>
+      </c>
+      <c r="E11" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D12" t="s">
+        <v>43</v>
+      </c>
+      <c r="E12" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>24</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D13" t="s">
+        <v>44</v>
+      </c>
+      <c r="E13" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D14" t="s">
+        <v>45</v>
+      </c>
+      <c r="E14" t="s">
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -933,4 +1040,85 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC441DD0-AAA7-4788-A5B0-1FD0AEA022F2}">
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16.5703125" customWidth="1"/>
+    <col min="2" max="2" width="19.7109375" customWidth="1"/>
+    <col min="3" max="3" width="59.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" t="s">
+        <v>45</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
done at my side
</commit_message>
<xml_diff>
--- a/src/test/resources/Templates/templateData.xlsx
+++ b/src/test/resources/Templates/templateData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Eclipse\ICEDQ\TestGenerator\src\test\resources\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED96965B-7EB8-417A-AF94-0AD39898A923}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D2EE0D1-7BDB-465C-8EE3-847669B40D2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Create template" sheetId="1" r:id="rId1"/>
@@ -153,25 +153,25 @@
     <t>My Pushdown template - using import template_Updated</t>
   </si>
   <si>
-    <t>My Checksum template - using dynamic template To delete</t>
-  </si>
-  <si>
-    <t>My Recon template - using dynamic template  To delete</t>
-  </si>
-  <si>
-    <t>My Validation template - using dynamic template  To delete</t>
-  </si>
-  <si>
-    <t>My Validation template - using import template  To delete</t>
-  </si>
-  <si>
-    <t>My Pushdown template - using import template  To delete</t>
-  </si>
-  <si>
     <t>My dynamic template  To delete</t>
   </si>
   <si>
     <t>My import template  To delete</t>
+  </si>
+  <si>
+    <t>My Checksum template - To delete</t>
+  </si>
+  <si>
+    <t>My Recon template - To delete</t>
+  </si>
+  <si>
+    <t>My Validation template - To delete</t>
+  </si>
+  <si>
+    <t>My Validation 01 template - To delete</t>
+  </si>
+  <si>
+    <t>My Pushdown template - To delete</t>
   </si>
 </sst>
 </file>
@@ -678,10 +678,10 @@
         <v>2</v>
       </c>
       <c r="D10" t="s">
+        <v>43</v>
+      </c>
+      <c r="E10" t="s">
         <v>41</v>
-      </c>
-      <c r="E10" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -695,10 +695,10 @@
         <v>3</v>
       </c>
       <c r="D11" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E11" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -712,10 +712,10 @@
         <v>4</v>
       </c>
       <c r="D12" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E12" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -729,10 +729,10 @@
         <v>27</v>
       </c>
       <c r="D13" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E13" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
@@ -746,10 +746,10 @@
         <v>28</v>
       </c>
       <c r="D14" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E14" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -1071,7 +1071,7 @@
         <v>12</v>
       </c>
       <c r="C2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -1082,7 +1082,7 @@
         <v>13</v>
       </c>
       <c r="C3" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -1093,7 +1093,7 @@
         <v>14</v>
       </c>
       <c r="C4" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -1104,7 +1104,7 @@
         <v>14</v>
       </c>
       <c r="C5" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -1115,7 +1115,7 @@
         <v>15</v>
       </c>
       <c r="C6" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>